<commit_message>
ci: add browserstack GH Actions workflow
</commit_message>
<xml_diff>
--- a/docs/test-cases/TestCases_2.0.xlsx
+++ b/docs/test-cases/TestCases_2.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\8t-wdio-appium-browserstack\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3359B5-819E-412B-888F-D416CDFE7324}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB73EE7-8E88-4E2A-9D3E-79A7BFD84C61}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -875,51 +875,176 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">1. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Username</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Password</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> fields were filled with example credentials
+      <t xml:space="preserve">1. Fill username and password with valid data
+2. Tap on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Login</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button
+3. Tap on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Change View</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button
+4. Add two products to cart
+5. Tap on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> icon
+6. Tap on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Checkout</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button
+7. Fill all mandatory fields of shipping information form
+8. Tap on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Continue</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button
+9. Verify products displayed on the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Overview</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> screen equal the added products
+10. Verify total amount was calculated including shipping tax
+11. Tap on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Finish</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The mandatory input fields were populated with valid data
 2. The </t>
     </r>
     <r>
@@ -1084,175 +1209,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> screen was opened</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Tap on the first example credentials
-2. Tap on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Login</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-3. Tap on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Change View</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-4. Add two products to cart
-5. Tap on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cart</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> icon
-6. Tap on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Checkout</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-7. Fill all mandatory fields of shipping information form
-8. Tap on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Continue</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-9. Verify products displayed on the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Overview</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> screen equal the added products
-10. Verify total amount was calculated including shipping tax
-11. Tap on </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Finish</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button</t>
     </r>
   </si>
 </sst>
@@ -1734,10 +1690,10 @@
         <v>18</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>6</v>

</xml_diff>